<commit_message>
update source docs and reparse data
</commit_message>
<xml_diff>
--- a/source-docs/TRIBES _ BONUSES.xlsx
+++ b/source-docs/TRIBES _ BONUSES.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="537">
   <si>
     <t>LAMIIRAN</t>
   </si>
@@ -324,15 +324,21 @@
     <t>WINTER'S VOICE</t>
   </si>
   <si>
-    <t>MILITANT BLOODLINE</t>
+    <t>MAGEHUNTER BLOODLINE</t>
   </si>
   <si>
     <t>(Spell) [6] Blast a wave of frost outward (3 Tile Width / Melee</t>
   </si>
   <si>
+    <t>Gain a permenant Lv.1 fire, water, electric, ice, wind, dark, or light</t>
+  </si>
+  <si>
     <t>range) dealing 1D8+SRV Ice DMG to all in range.</t>
   </si>
   <si>
+    <t>resistance.</t>
+  </si>
+  <si>
     <t>GOTHRIN</t>
   </si>
   <si>
@@ -618,7 +624,7 @@
     <t>Agoraaz, M'edu, Tuael'va</t>
   </si>
   <si>
-    <t>wraps alongsize others with bright, gold-adorned suits.</t>
+    <t>wraps alongside others with bright, gold-adorned suits.</t>
   </si>
   <si>
     <t>Mezzirth, Axava, B'nelva</t>
@@ -1086,7 +1092,7 @@
     <t>usually required Attribute threshold.</t>
   </si>
   <si>
-    <t>deals 1D6+STR slash / pierce DMG (type chosen is permenant)</t>
+    <t>deals 1D6+STR slash / pierce DMG (type chosen is permanent)</t>
   </si>
   <si>
     <t>WINGED RISE</t>
@@ -3510,7 +3516,9 @@
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
-      <c r="F45" s="72"/>
+      <c r="F45" s="72" t="s">
+        <v>103</v>
+      </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
       <c r="I45" s="16"/>
@@ -3522,13 +3530,15 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
-      <c r="F46" s="76"/>
+      <c r="F46" s="76" t="s">
+        <v>105</v>
+      </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
       <c r="I46" s="77"/>
@@ -3712,7 +3722,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -3743,7 +3753,7 @@
     </row>
     <row r="3">
       <c r="A3" s="83" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -3754,13 +3764,13 @@
         <v>-1.0</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="84" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -3771,13 +3781,13 @@
         <v>4</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="84" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -3788,13 +3798,13 @@
         <v>4</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="84" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -3805,13 +3815,13 @@
         <v>1.0</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="84" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -3822,13 +3832,13 @@
         <v>1.0</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="84" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -3839,13 +3849,13 @@
         <v>-1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="84" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -3856,13 +3866,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="84" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -3877,18 +3887,18 @@
     </row>
     <row r="11">
       <c r="A11" s="84" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="84" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -3900,13 +3910,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="85" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -3920,7 +3930,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -3955,7 +3965,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -3975,7 +3985,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -3989,13 +3999,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -4015,7 +4025,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -4035,7 +4045,7 @@
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -4051,7 +4061,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -4061,20 +4071,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -4087,20 +4097,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24">
@@ -4150,14 +4160,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -4170,14 +4180,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -4195,7 +4205,7 @@
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -4218,14 +4228,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -4238,14 +4248,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -4284,14 +4294,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -4304,14 +4314,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -4324,7 +4334,7 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
@@ -4352,14 +4362,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -4372,14 +4382,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -4392,14 +4402,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -4431,7 +4441,7 @@
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -4444,14 +4454,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -4469,7 +4479,7 @@
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -4654,7 +4664,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -4685,7 +4695,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -4696,13 +4706,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -4713,13 +4723,13 @@
         <v>1.0</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -4730,13 +4740,13 @@
         <v>4</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -4751,7 +4761,7 @@
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -4762,13 +4772,13 @@
         <v>4</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -4779,13 +4789,13 @@
         <v>4</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -4796,13 +4806,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -4813,24 +4823,24 @@
         <v>-1.0</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="K10" s="25"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -4842,13 +4852,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -4862,7 +4872,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -4897,7 +4907,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -4917,7 +4927,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -4931,13 +4941,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -4957,7 +4967,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -4971,13 +4981,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -4993,7 +5003,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -5003,20 +5013,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -5029,20 +5039,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24">
@@ -5092,14 +5102,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -5112,14 +5122,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -5132,14 +5142,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -5162,14 +5172,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -5182,14 +5192,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -5207,7 +5217,7 @@
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -5230,14 +5240,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -5250,14 +5260,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -5275,7 +5285,7 @@
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -5305,7 +5315,7 @@
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -5325,7 +5335,7 @@
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -5343,7 +5353,7 @@
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -5368,14 +5378,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -5388,14 +5398,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -5413,7 +5423,7 @@
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -5596,7 +5606,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -5627,7 +5637,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -5638,13 +5648,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -5655,13 +5665,13 @@
         <v>-1.0</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -5672,13 +5682,13 @@
         <v>4</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -5689,13 +5699,13 @@
         <v>4</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -5706,13 +5716,13 @@
         <v>1.0</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -5723,13 +5733,13 @@
         <v>1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -5740,13 +5750,13 @@
         <v>-1.0</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -5757,24 +5767,24 @@
         <v>4</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="K10" s="25"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -5786,13 +5796,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -5806,7 +5816,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -5821,7 +5831,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -5843,7 +5853,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -5863,7 +5873,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -5877,13 +5887,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -5903,7 +5913,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -5917,13 +5927,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -5939,7 +5949,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -5949,20 +5959,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -5975,20 +5985,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="24">
@@ -6038,14 +6048,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -6058,14 +6068,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -6078,7 +6088,7 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
@@ -6113,7 +6123,7 @@
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -6133,7 +6143,7 @@
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -6151,7 +6161,7 @@
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -6174,14 +6184,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -6194,14 +6204,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -6214,14 +6224,14 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -6244,14 +6254,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -6264,14 +6274,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -6284,14 +6294,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -6316,7 +6326,7 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
@@ -6334,7 +6344,7 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
@@ -6352,7 +6362,7 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
@@ -6538,7 +6548,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -6569,7 +6579,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -6580,13 +6590,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -6597,13 +6607,13 @@
         <v>-1.0</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -6614,13 +6624,13 @@
         <v>-1.0</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -6631,13 +6641,13 @@
         <v>4</v>
       </c>
       <c r="J6" s="24" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="K6" s="25"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -6648,13 +6658,13 @@
         <v>4</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -6665,13 +6675,13 @@
         <v>1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -6682,13 +6692,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -6699,24 +6709,24 @@
         <v>4</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="K10" s="25"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -6728,7 +6738,7 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="K12" s="23"/>
     </row>
@@ -6746,7 +6756,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -6761,7 +6771,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -6783,7 +6793,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -6803,7 +6813,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -6811,19 +6821,19 @@
         <v>50</v>
       </c>
       <c r="G17" s="41" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="H17" s="35" t="s">
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -6843,7 +6853,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -6857,13 +6867,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -6879,7 +6889,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -6889,20 +6899,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -6915,20 +6925,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24">
@@ -6978,14 +6988,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -6998,14 +7008,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -7018,14 +7028,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -7048,14 +7058,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -7068,14 +7078,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -7093,7 +7103,7 @@
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -7116,14 +7126,14 @@
     </row>
     <row r="36">
       <c r="A36" s="67" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -7136,14 +7146,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -7156,7 +7166,7 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
@@ -7184,14 +7194,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -7204,14 +7214,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -7224,14 +7234,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -7256,14 +7266,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -7276,14 +7286,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -7296,7 +7306,7 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
@@ -7483,7 +7493,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -7514,7 +7524,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -7525,13 +7535,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -7542,13 +7552,13 @@
         <v>4</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -7559,13 +7569,13 @@
         <v>1.0</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -7576,13 +7586,13 @@
         <v>-1.0</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -7593,13 +7603,13 @@
         <v>4</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -7610,13 +7620,13 @@
         <v>-1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -7627,13 +7637,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -7644,24 +7654,24 @@
         <v>4</v>
       </c>
       <c r="J10" s="93" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="K10" s="27"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -7673,13 +7683,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -7693,7 +7703,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -7708,7 +7718,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -7730,7 +7740,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -7750,7 +7760,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -7758,19 +7768,19 @@
         <v>50</v>
       </c>
       <c r="G17" s="41" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="H17" s="35" t="s">
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -7790,7 +7800,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -7804,13 +7814,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -7826,7 +7836,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -7836,20 +7846,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -7862,20 +7872,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24">
@@ -7925,14 +7935,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -7945,14 +7955,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -7965,14 +7975,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -7995,14 +8005,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -8015,14 +8025,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -8035,14 +8045,14 @@
     </row>
     <row r="34">
       <c r="A34" s="73" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B34" s="74"/>
       <c r="C34" s="74"/>
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -8065,14 +8075,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -8085,14 +8095,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -8105,14 +8115,14 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -8135,14 +8145,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -8155,14 +8165,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -8175,14 +8185,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -8207,14 +8217,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -8227,14 +8237,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -8247,14 +8257,14 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -8437,7 +8447,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -8456,7 +8466,7 @@
       <c r="B2" s="9"/>
       <c r="C2" s="10"/>
       <c r="F2" s="13" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="G2" s="14"/>
       <c r="J2" s="13" t="s">
@@ -8466,7 +8476,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -8474,16 +8484,16 @@
         <v>3</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -8491,16 +8501,16 @@
         <v>7</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -8508,16 +8518,16 @@
         <v>10</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -8525,16 +8535,16 @@
         <v>13</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J6" s="94" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -8542,16 +8552,16 @@
         <v>16</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -8559,16 +8569,16 @@
         <v>19</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -8576,16 +8586,16 @@
         <v>22</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -8593,16 +8603,16 @@
         <v>25</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J10" s="94" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="K10" s="27"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
@@ -8610,16 +8620,16 @@
         <v>28</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="J11" s="95" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="K11" s="3"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -8631,13 +8641,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="96" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="K12" s="21"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -8651,7 +8661,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="96" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="K13" s="21"/>
     </row>
@@ -8666,7 +8676,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="96" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="K14" s="21"/>
     </row>
@@ -8686,13 +8696,13 @@
         <v>38</v>
       </c>
       <c r="J15" s="96" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="K15" s="21"/>
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -8706,13 +8716,13 @@
         <v>47</v>
       </c>
       <c r="J16" s="97" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="K16" s="17"/>
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -8726,13 +8736,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="96" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="K17" s="21"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -8746,13 +8756,13 @@
         <v>56</v>
       </c>
       <c r="J18" s="96" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="K18" s="21"/>
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -8766,13 +8776,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="96" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="K19" s="21"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -8780,13 +8790,13 @@
       <c r="G20" s="44"/>
       <c r="H20" s="44"/>
       <c r="J20" s="96" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="K20" s="21"/>
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -8796,39 +8806,39 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="96" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="K21" s="21"/>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
       <c r="J22" s="96" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="K22" s="21"/>
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="96" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="K23" s="21"/>
     </row>
@@ -8839,7 +8849,7 @@
       <c r="F24" s="43"/>
       <c r="G24" s="59"/>
       <c r="J24" s="96" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="K24" s="21"/>
     </row>
@@ -8856,7 +8866,7 @@
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="96" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="K25" s="21"/>
       <c r="L25" s="61"/>
@@ -8876,13 +8886,13 @@
       <c r="H26" s="47"/>
       <c r="I26" s="48"/>
       <c r="J26" s="96" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="K26" s="21"/>
     </row>
     <row r="27">
       <c r="J27" s="98" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="K27" s="32"/>
       <c r="L27" s="63"/>
@@ -8891,14 +8901,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -8911,14 +8921,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -8931,14 +8941,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -8961,14 +8971,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -8981,14 +8991,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -9001,14 +9011,14 @@
     </row>
     <row r="34">
       <c r="A34" s="73" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B34" s="74"/>
       <c r="C34" s="74"/>
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -9031,14 +9041,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -9051,14 +9061,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -9071,14 +9081,14 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -9101,14 +9111,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -9121,14 +9131,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -9141,14 +9151,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -9180,7 +9190,7 @@
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -9200,7 +9210,7 @@
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -9218,7 +9228,7 @@
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -9458,7 +9468,7 @@
       </c>
       <c r="G3" s="12"/>
       <c r="J3" s="18" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="K3" s="5"/>
     </row>
@@ -9504,7 +9514,7 @@
       </c>
       <c r="G7" s="12"/>
       <c r="J7" s="18" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="K7" s="5"/>
     </row>
@@ -9546,7 +9556,7 @@
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="K11" s="5"/>
     </row>
@@ -9760,14 +9770,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -9822,14 +9832,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -9884,14 +9894,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -9946,14 +9956,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -10010,14 +10020,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -10232,19 +10242,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="106" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B1" s="107"/>
       <c r="C1" s="106" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D1" s="107"/>
       <c r="E1" s="106" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F1" s="107"/>
       <c r="G1" s="106" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="I1" s="108"/>
       <c r="K1" s="108"/>
@@ -10262,19 +10272,19 @@
     </row>
     <row r="3">
       <c r="A3" s="110" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B3" s="107"/>
       <c r="C3" s="111" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D3" s="107"/>
       <c r="E3" s="111" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F3" s="107"/>
       <c r="G3" s="111" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="I3" s="112"/>
       <c r="K3" s="112"/>
@@ -10334,19 +10344,19 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B9" s="107"/>
       <c r="C9" s="106" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D9" s="107"/>
       <c r="E9" s="106" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F9" s="107"/>
       <c r="G9" s="106" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="I9" s="108"/>
       <c r="K9" s="108"/>
@@ -10364,19 +10374,19 @@
     </row>
     <row r="11">
       <c r="A11" s="111" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B11" s="107"/>
       <c r="C11" s="111" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D11" s="107"/>
       <c r="E11" s="111" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="F11" s="107"/>
       <c r="G11" s="110" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="I11" s="112"/>
       <c r="K11" s="112"/>
@@ -10436,19 +10446,19 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B17" s="107"/>
       <c r="C17" s="106" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D17" s="107"/>
       <c r="E17" s="106" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F17" s="107"/>
       <c r="G17" s="106" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="I17" s="108"/>
       <c r="K17" s="108"/>
@@ -10466,19 +10476,19 @@
     </row>
     <row r="19">
       <c r="A19" s="111" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B19" s="107"/>
       <c r="C19" s="114" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D19" s="107"/>
       <c r="E19" s="111" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F19" s="107"/>
       <c r="G19" s="111" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="I19" s="112"/>
       <c r="K19" s="112"/>
@@ -10538,19 +10548,19 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B25" s="107"/>
       <c r="C25" s="106" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D25" s="107"/>
       <c r="E25" s="106" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F25" s="107"/>
       <c r="G25" s="106" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="I25" s="108"/>
       <c r="K25" s="108"/>
@@ -10568,19 +10578,19 @@
     </row>
     <row r="27">
       <c r="A27" s="114" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B27" s="107"/>
       <c r="C27" s="114" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D27" s="107"/>
       <c r="E27" s="111" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F27" s="107"/>
       <c r="G27" s="114" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="I27" s="112"/>
       <c r="K27" s="112"/>

</xml_diff>

<commit_message>
update source docs, reparse all, update medic talent description
</commit_message>
<xml_diff>
--- a/source-docs/TRIBES _ BONUSES.xlsx
+++ b/source-docs/TRIBES _ BONUSES.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="538">
   <si>
     <t>LAMIIRAN</t>
   </si>
@@ -337,6 +337,9 @@
   </si>
   <si>
     <t>resistance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
   <si>
     <t>GOTHRIN</t>
@@ -1468,10 +1471,10 @@
     <t>Inanimate (no Spiritual Influence)</t>
   </si>
   <si>
-    <t>- Can not use consumables or heal</t>
-  </si>
-  <si>
-    <t>from cooking / potions</t>
+    <t>- Can throw themselves as their</t>
+  </si>
+  <si>
+    <t>MOVE action and reappear at target</t>
   </si>
   <si>
     <t>BOND ENHANCEMENT</t>
@@ -1504,7 +1507,7 @@
     <t>(Ability) While in inanimate form strike a target (5 tile range; advantage</t>
   </si>
   <si>
-    <t>Lv.1 resistance (armor)</t>
+    <t>Lv.2 resistance (armor)</t>
   </si>
   <si>
     <t>on ATK: weapon DMG or 1D6+STR crush) can end inanimate form.</t>
@@ -3546,7 +3549,9 @@
       <c r="K46" s="78"/>
       <c r="L46" s="64"/>
       <c r="M46" s="64"/>
-      <c r="N46" s="64"/>
+      <c r="N46" s="64" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="81"/>
@@ -3722,7 +3727,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -3753,7 +3758,7 @@
     </row>
     <row r="3">
       <c r="A3" s="83" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -3764,13 +3769,13 @@
         <v>-1.0</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="84" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -3781,13 +3786,13 @@
         <v>4</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="84" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -3798,13 +3803,13 @@
         <v>4</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="84" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -3815,13 +3820,13 @@
         <v>1.0</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="84" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -3832,13 +3837,13 @@
         <v>1.0</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="84" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -3849,13 +3854,13 @@
         <v>-1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="84" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -3866,13 +3871,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="84" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -3887,18 +3892,18 @@
     </row>
     <row r="11">
       <c r="A11" s="84" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="84" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -3910,13 +3915,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="85" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -3930,7 +3935,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -3965,7 +3970,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -3985,7 +3990,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -3999,13 +4004,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -4025,7 +4030,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -4045,7 +4050,7 @@
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -4061,7 +4066,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -4071,20 +4076,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -4097,20 +4102,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24">
@@ -4160,14 +4165,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -4180,14 +4185,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -4205,7 +4210,7 @@
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -4228,14 +4233,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -4248,14 +4253,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -4294,14 +4299,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -4314,14 +4319,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -4334,7 +4339,7 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
@@ -4362,14 +4367,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -4382,14 +4387,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -4402,14 +4407,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -4441,7 +4446,7 @@
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -4454,14 +4459,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -4479,7 +4484,7 @@
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -4664,7 +4669,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -4695,7 +4700,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -4706,13 +4711,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -4723,13 +4728,13 @@
         <v>1.0</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -4740,13 +4745,13 @@
         <v>4</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -4761,7 +4766,7 @@
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -4772,13 +4777,13 @@
         <v>4</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -4789,13 +4794,13 @@
         <v>4</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -4806,13 +4811,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -4823,24 +4828,24 @@
         <v>-1.0</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K10" s="25"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -4852,13 +4857,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -4872,7 +4877,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -4907,7 +4912,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -4927,7 +4932,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -4941,13 +4946,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -4967,7 +4972,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -4981,13 +4986,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -5003,7 +5008,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -5013,20 +5018,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -5039,20 +5044,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24">
@@ -5102,14 +5107,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -5122,14 +5127,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -5142,14 +5147,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -5172,14 +5177,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -5192,14 +5197,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -5217,7 +5222,7 @@
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -5240,14 +5245,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -5260,14 +5265,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -5285,7 +5290,7 @@
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -5315,7 +5320,7 @@
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -5335,7 +5340,7 @@
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -5353,7 +5358,7 @@
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -5378,14 +5383,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -5398,14 +5403,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -5423,7 +5428,7 @@
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -5606,7 +5611,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -5637,7 +5642,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -5648,13 +5653,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -5665,13 +5670,13 @@
         <v>-1.0</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -5682,13 +5687,13 @@
         <v>4</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -5699,13 +5704,13 @@
         <v>4</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -5716,13 +5721,13 @@
         <v>1.0</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -5733,13 +5738,13 @@
         <v>1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -5750,13 +5755,13 @@
         <v>-1.0</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -5767,24 +5772,24 @@
         <v>4</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K10" s="25"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -5796,13 +5801,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -5816,7 +5821,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -5831,7 +5836,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -5853,7 +5858,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -5873,7 +5878,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -5887,13 +5892,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -5913,7 +5918,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -5927,13 +5932,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -5949,7 +5954,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -5959,20 +5964,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -5985,20 +5990,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="24">
@@ -6048,14 +6053,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -6068,14 +6073,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -6088,7 +6093,7 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
@@ -6123,7 +6128,7 @@
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -6143,7 +6148,7 @@
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -6161,7 +6166,7 @@
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -6184,14 +6189,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -6204,14 +6209,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -6224,14 +6229,14 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -6254,14 +6259,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -6274,14 +6279,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -6294,14 +6299,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -6326,7 +6331,7 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
@@ -6344,7 +6349,7 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
@@ -6362,7 +6367,7 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
@@ -6548,7 +6553,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -6579,7 +6584,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -6590,13 +6595,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -6607,13 +6612,13 @@
         <v>-1.0</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -6624,13 +6629,13 @@
         <v>-1.0</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -6641,13 +6646,13 @@
         <v>4</v>
       </c>
       <c r="J6" s="24" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="K6" s="25"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -6658,13 +6663,13 @@
         <v>4</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -6675,13 +6680,13 @@
         <v>1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -6692,13 +6697,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -6709,24 +6714,24 @@
         <v>4</v>
       </c>
       <c r="J10" s="24" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="K10" s="25"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -6738,7 +6743,7 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="K12" s="23"/>
     </row>
@@ -6756,7 +6761,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -6771,7 +6776,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -6793,7 +6798,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -6813,7 +6818,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -6821,19 +6826,19 @@
         <v>50</v>
       </c>
       <c r="G17" s="41" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H17" s="35" t="s">
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -6853,7 +6858,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -6867,13 +6872,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -6889,7 +6894,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -6899,20 +6904,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -6925,20 +6930,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24">
@@ -6988,14 +6993,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -7008,14 +7013,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -7028,14 +7033,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -7058,14 +7063,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -7078,14 +7083,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -7103,7 +7108,7 @@
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -7126,14 +7131,14 @@
     </row>
     <row r="36">
       <c r="A36" s="67" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -7146,14 +7151,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -7166,7 +7171,7 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
@@ -7194,14 +7199,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -7214,14 +7219,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -7234,14 +7239,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -7266,14 +7271,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -7286,14 +7291,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -7306,7 +7311,7 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
@@ -7493,7 +7498,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -7524,7 +7529,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -7535,13 +7540,13 @@
         <v>4</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -7552,13 +7557,13 @@
         <v>4</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -7569,13 +7574,13 @@
         <v>1.0</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -7586,13 +7591,13 @@
         <v>-1.0</v>
       </c>
       <c r="J6" s="26" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -7603,13 +7608,13 @@
         <v>4</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -7620,13 +7625,13 @@
         <v>-1.0</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -7637,13 +7642,13 @@
         <v>4</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -7654,24 +7659,24 @@
         <v>4</v>
       </c>
       <c r="J10" s="93" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K10" s="27"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K11" s="5"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -7683,13 +7688,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K12" s="23"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -7703,7 +7708,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="24" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="K13" s="25"/>
     </row>
@@ -7718,7 +7723,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="24" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="K14" s="25"/>
     </row>
@@ -7740,7 +7745,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -7760,7 +7765,7 @@
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -7768,19 +7773,19 @@
         <v>50</v>
       </c>
       <c r="G17" s="41" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H17" s="35" t="s">
         <v>52</v>
       </c>
       <c r="J17" s="42" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K17" s="14"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -7800,7 +7805,7 @@
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -7814,13 +7819,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="42" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K19" s="14"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -7836,7 +7841,7 @@
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -7846,20 +7851,20 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="49" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K21" s="50" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
@@ -7872,20 +7877,20 @@
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="56" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K23" s="57" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="24">
@@ -7935,14 +7940,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -7955,14 +7960,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -7975,14 +7980,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -8005,14 +8010,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -8025,14 +8030,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -8045,14 +8050,14 @@
     </row>
     <row r="34">
       <c r="A34" s="73" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B34" s="74"/>
       <c r="C34" s="74"/>
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -8075,14 +8080,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -8095,14 +8100,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -8115,14 +8120,14 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -8145,14 +8150,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -8165,14 +8170,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -8185,14 +8190,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -8217,14 +8222,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -8237,14 +8242,14 @@
     </row>
     <row r="45">
       <c r="A45" s="69" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -8257,14 +8262,14 @@
     </row>
     <row r="46">
       <c r="A46" s="73" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B46" s="74"/>
       <c r="C46" s="74"/>
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -8447,7 +8452,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
@@ -8466,7 +8471,7 @@
       <c r="B2" s="9"/>
       <c r="C2" s="10"/>
       <c r="F2" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G2" s="14"/>
       <c r="J2" s="13" t="s">
@@ -8476,7 +8481,7 @@
     </row>
     <row r="3">
       <c r="A3" s="15" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="17"/>
@@ -8484,16 +8489,16 @@
         <v>3</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B4" s="20"/>
       <c r="C4" s="21"/>
@@ -8501,16 +8506,16 @@
         <v>7</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K4" s="23"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B5" s="20"/>
       <c r="C5" s="21"/>
@@ -8518,16 +8523,16 @@
         <v>10</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J5" s="24" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K5" s="25"/>
     </row>
     <row r="6">
       <c r="A6" s="19" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B6" s="20"/>
       <c r="C6" s="21"/>
@@ -8535,16 +8540,16 @@
         <v>13</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J6" s="94" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K6" s="27"/>
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B7" s="20"/>
       <c r="C7" s="21"/>
@@ -8552,16 +8557,16 @@
         <v>16</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K7" s="5"/>
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21"/>
@@ -8569,16 +8574,16 @@
         <v>19</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K8" s="23"/>
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="21"/>
@@ -8586,16 +8591,16 @@
         <v>22</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="K9" s="25"/>
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B10" s="20"/>
       <c r="C10" s="21"/>
@@ -8603,16 +8608,16 @@
         <v>25</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J10" s="94" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K10" s="27"/>
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
@@ -8620,16 +8625,16 @@
         <v>28</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J11" s="95" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K11" s="3"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="21"/>
@@ -8641,13 +8646,13 @@
         <v>34</v>
       </c>
       <c r="J12" s="96" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="K12" s="21"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="32"/>
@@ -8661,7 +8666,7 @@
         <v>38</v>
       </c>
       <c r="J13" s="96" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K13" s="21"/>
     </row>
@@ -8676,7 +8681,7 @@
         <v>41</v>
       </c>
       <c r="J14" s="96" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K14" s="21"/>
     </row>
@@ -8696,13 +8701,13 @@
         <v>38</v>
       </c>
       <c r="J15" s="96" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="K15" s="21"/>
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="23"/>
@@ -8716,13 +8721,13 @@
         <v>47</v>
       </c>
       <c r="J16" s="97" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K16" s="17"/>
     </row>
     <row r="17">
       <c r="A17" s="39" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B17" s="20"/>
       <c r="C17" s="25"/>
@@ -8736,13 +8741,13 @@
         <v>52</v>
       </c>
       <c r="J17" s="96" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="K17" s="21"/>
     </row>
     <row r="18">
       <c r="A18" s="39" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B18" s="20"/>
       <c r="C18" s="25"/>
@@ -8756,13 +8761,13 @@
         <v>56</v>
       </c>
       <c r="J18" s="96" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K18" s="21"/>
     </row>
     <row r="19">
       <c r="A19" s="39" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B19" s="20"/>
       <c r="C19" s="25"/>
@@ -8776,13 +8781,13 @@
         <v>60</v>
       </c>
       <c r="J19" s="96" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="K19" s="21"/>
     </row>
     <row r="20">
       <c r="A20" s="39" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="25"/>
@@ -8790,13 +8795,13 @@
       <c r="G20" s="44"/>
       <c r="H20" s="44"/>
       <c r="J20" s="96" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K20" s="21"/>
     </row>
     <row r="21">
       <c r="A21" s="39" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="25"/>
@@ -8806,39 +8811,39 @@
       <c r="G21" s="47"/>
       <c r="H21" s="48"/>
       <c r="J21" s="96" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K21" s="21"/>
     </row>
     <row r="22">
       <c r="A22" s="39" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="25"/>
       <c r="F22" s="51" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G22" s="16"/>
       <c r="H22" s="23"/>
       <c r="J22" s="96" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="K22" s="21"/>
     </row>
     <row r="23">
       <c r="A23" s="53" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B23" s="54"/>
       <c r="C23" s="27"/>
       <c r="F23" s="55" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="G23" s="20"/>
       <c r="H23" s="25"/>
       <c r="J23" s="96" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K23" s="21"/>
     </row>
@@ -8849,7 +8854,7 @@
       <c r="F24" s="43"/>
       <c r="G24" s="59"/>
       <c r="J24" s="96" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="K24" s="21"/>
     </row>
@@ -8866,7 +8871,7 @@
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="96" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K25" s="21"/>
       <c r="L25" s="61"/>
@@ -8886,13 +8891,13 @@
       <c r="H26" s="47"/>
       <c r="I26" s="48"/>
       <c r="J26" s="96" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K26" s="21"/>
     </row>
     <row r="27">
       <c r="J27" s="98" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K27" s="32"/>
       <c r="L27" s="63"/>
@@ -8901,14 +8906,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -8921,14 +8926,14 @@
     </row>
     <row r="29">
       <c r="A29" s="69" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="70"/>
       <c r="E29" s="71"/>
       <c r="F29" s="72" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
@@ -8941,14 +8946,14 @@
     </row>
     <row r="30">
       <c r="A30" s="73" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B30" s="74"/>
       <c r="C30" s="74"/>
       <c r="D30" s="75"/>
       <c r="E30" s="71"/>
       <c r="F30" s="76" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="G30" s="77"/>
       <c r="H30" s="77"/>
@@ -8971,14 +8976,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -8991,14 +8996,14 @@
     </row>
     <row r="33">
       <c r="A33" s="69" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
       <c r="D33" s="70"/>
       <c r="E33" s="71"/>
       <c r="F33" s="72" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="G33" s="16"/>
       <c r="H33" s="16"/>
@@ -9011,14 +9016,14 @@
     </row>
     <row r="34">
       <c r="A34" s="73" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B34" s="74"/>
       <c r="C34" s="74"/>
       <c r="D34" s="75"/>
       <c r="E34" s="71"/>
       <c r="F34" s="76" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G34" s="77"/>
       <c r="H34" s="77"/>
@@ -9041,14 +9046,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -9061,14 +9066,14 @@
     </row>
     <row r="37">
       <c r="A37" s="69" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
       <c r="D37" s="70"/>
       <c r="E37" s="71"/>
       <c r="F37" s="72" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="G37" s="16"/>
       <c r="H37" s="16"/>
@@ -9081,14 +9086,14 @@
     </row>
     <row r="38">
       <c r="A38" s="73" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B38" s="74"/>
       <c r="C38" s="74"/>
       <c r="D38" s="75"/>
       <c r="E38" s="71"/>
       <c r="F38" s="76" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G38" s="77"/>
       <c r="H38" s="77"/>
@@ -9111,14 +9116,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -9131,14 +9136,14 @@
     </row>
     <row r="41">
       <c r="A41" s="69" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
       <c r="D41" s="70"/>
       <c r="E41" s="71"/>
       <c r="F41" s="72" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G41" s="16"/>
       <c r="H41" s="16"/>
@@ -9151,14 +9156,14 @@
     </row>
     <row r="42">
       <c r="A42" s="73" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B42" s="74"/>
       <c r="C42" s="74"/>
       <c r="D42" s="75"/>
       <c r="E42" s="71"/>
       <c r="F42" s="76" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="G42" s="77"/>
       <c r="H42" s="77"/>
@@ -9190,7 +9195,7 @@
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -9210,7 +9215,7 @@
       <c r="D45" s="70"/>
       <c r="E45" s="71"/>
       <c r="F45" s="72" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="16"/>
@@ -9228,7 +9233,7 @@
       <c r="D46" s="75"/>
       <c r="E46" s="71"/>
       <c r="F46" s="76" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="G46" s="77"/>
       <c r="H46" s="77"/>
@@ -9468,7 +9473,7 @@
       </c>
       <c r="G3" s="12"/>
       <c r="J3" s="18" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K3" s="5"/>
     </row>
@@ -9514,7 +9519,7 @@
       </c>
       <c r="G7" s="12"/>
       <c r="J7" s="18" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K7" s="5"/>
     </row>
@@ -9556,7 +9561,7 @@
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="J11" s="18" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="K11" s="5"/>
     </row>
@@ -9770,14 +9775,14 @@
     </row>
     <row r="28">
       <c r="A28" s="65" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
       <c r="D28" s="48"/>
       <c r="E28" s="66"/>
       <c r="F28" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G28" s="47"/>
       <c r="H28" s="47"/>
@@ -9832,14 +9837,14 @@
     </row>
     <row r="32">
       <c r="A32" s="65" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="47"/>
       <c r="D32" s="48"/>
       <c r="E32" s="66"/>
       <c r="F32" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G32" s="47"/>
       <c r="H32" s="47"/>
@@ -9894,14 +9899,14 @@
     </row>
     <row r="36">
       <c r="A36" s="65" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="47"/>
       <c r="D36" s="48"/>
       <c r="E36" s="66"/>
       <c r="F36" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G36" s="47"/>
       <c r="H36" s="47"/>
@@ -9956,14 +9961,14 @@
     </row>
     <row r="40">
       <c r="A40" s="65" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B40" s="47"/>
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="66"/>
       <c r="F40" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G40" s="47"/>
       <c r="H40" s="47"/>
@@ -10020,14 +10025,14 @@
     </row>
     <row r="44">
       <c r="A44" s="65" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B44" s="47"/>
       <c r="C44" s="47"/>
       <c r="D44" s="48"/>
       <c r="E44" s="66"/>
       <c r="F44" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G44" s="47"/>
       <c r="H44" s="47"/>
@@ -10242,19 +10247,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="106" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B1" s="107"/>
       <c r="C1" s="106" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D1" s="107"/>
       <c r="E1" s="106" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F1" s="107"/>
       <c r="G1" s="106" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="I1" s="108"/>
       <c r="K1" s="108"/>
@@ -10272,19 +10277,19 @@
     </row>
     <row r="3">
       <c r="A3" s="110" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B3" s="107"/>
       <c r="C3" s="111" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D3" s="107"/>
       <c r="E3" s="111" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F3" s="107"/>
       <c r="G3" s="111" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="I3" s="112"/>
       <c r="K3" s="112"/>
@@ -10344,19 +10349,19 @@
     </row>
     <row r="9">
       <c r="A9" s="106" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B9" s="107"/>
       <c r="C9" s="106" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D9" s="107"/>
       <c r="E9" s="106" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F9" s="107"/>
       <c r="G9" s="106" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="I9" s="108"/>
       <c r="K9" s="108"/>
@@ -10374,19 +10379,19 @@
     </row>
     <row r="11">
       <c r="A11" s="111" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B11" s="107"/>
       <c r="C11" s="111" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D11" s="107"/>
       <c r="E11" s="111" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F11" s="107"/>
       <c r="G11" s="110" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="I11" s="112"/>
       <c r="K11" s="112"/>
@@ -10446,19 +10451,19 @@
     </row>
     <row r="17">
       <c r="A17" s="106" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B17" s="107"/>
       <c r="C17" s="106" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="D17" s="107"/>
       <c r="E17" s="106" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F17" s="107"/>
       <c r="G17" s="106" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="I17" s="108"/>
       <c r="K17" s="108"/>
@@ -10476,19 +10481,19 @@
     </row>
     <row r="19">
       <c r="A19" s="111" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B19" s="107"/>
       <c r="C19" s="114" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D19" s="107"/>
       <c r="E19" s="111" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F19" s="107"/>
       <c r="G19" s="111" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="I19" s="112"/>
       <c r="K19" s="112"/>
@@ -10548,19 +10553,19 @@
     </row>
     <row r="25">
       <c r="A25" s="106" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B25" s="107"/>
       <c r="C25" s="106" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D25" s="107"/>
       <c r="E25" s="106" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F25" s="107"/>
       <c r="G25" s="106" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="I25" s="108"/>
       <c r="K25" s="108"/>
@@ -10578,19 +10583,19 @@
     </row>
     <row r="27">
       <c r="A27" s="114" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B27" s="107"/>
       <c r="C27" s="114" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="D27" s="107"/>
       <c r="E27" s="111" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F27" s="107"/>
       <c r="G27" s="114" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="I27" s="112"/>
       <c r="K27" s="112"/>

</xml_diff>